<commit_message>
All new tookit and email verification
</commit_message>
<xml_diff>
--- a/AdvanceCRM/AdvanceCRM.Web/Templates/ClientSupression_Template.xlsx
+++ b/AdvanceCRM/AdvanceCRM.Web/Templates/ClientSupression_Template.xlsx
@@ -12,15 +12,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
-    <t>CompanyName</t>
+    <t>Sr No</t>
   </si>
   <si>
-    <t>FirstName</t>
+    <t>Company Name</t>
   </si>
   <si>
-    <t>LastName</t>
+    <t>First Name</t>
+  </si>
+  <si>
+    <t>Last Name</t>
   </si>
   <si>
     <t>Email</t>
@@ -81,15 +84,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.488309860229492" customWidth="1"/>
-    <col min="2" max="2" width="9.923392295837402" customWidth="1"/>
-    <col min="3" max="3" width="9.6134033203125" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -111,6 +115,9 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <headerFooter/>

</xml_diff>

<commit_message>
toolkit import template updated
</commit_message>
<xml_diff>
--- a/AdvanceCRM/AdvanceCRM.Web/Templates/ClientSupression_Template.xlsx
+++ b/AdvanceCRM/AdvanceCRM.Web/Templates/ClientSupression_Template.xlsx
@@ -12,9 +12,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Sr No</t>
+  </si>
+  <si>
+    <t>Master Account Id</t>
+  </si>
+  <si>
+    <t>Campaign Id</t>
   </si>
   <si>
     <t>Company Name</t>
@@ -84,7 +90,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -94,6 +100,8 @@
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -118,6 +126,12 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
   <headerFooter/>

</xml_diff>